<commit_message>
fix: Rango en commandos corregido
</commit_message>
<xml_diff>
--- a/1toolConverter_local/backend/Dixell/tablas_extraidas.xlsx
+++ b/1toolConverter_local/backend/Dixell/tablas_extraidas.xlsx
@@ -12251,7 +12251,7 @@
         <v>0</v>
       </c>
       <c r="L116" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M116" t="inlineStr"/>
       <c r="N116" t="n">
@@ -12355,7 +12355,7 @@
         <v>0</v>
       </c>
       <c r="L117" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M117" t="inlineStr"/>
       <c r="N117" t="n">
@@ -12459,7 +12459,7 @@
         <v>0</v>
       </c>
       <c r="L118" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M118" t="inlineStr"/>
       <c r="N118" t="n">
@@ -12563,7 +12563,7 @@
         <v>0</v>
       </c>
       <c r="L119" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M119" t="inlineStr"/>
       <c r="N119" t="n">
@@ -12667,7 +12667,7 @@
         <v>0</v>
       </c>
       <c r="L120" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M120" t="inlineStr"/>
       <c r="N120" t="n">
@@ -12771,7 +12771,7 @@
         <v>0</v>
       </c>
       <c r="L121" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M121" t="inlineStr"/>
       <c r="N121" t="n">
@@ -12875,7 +12875,7 @@
         <v>0</v>
       </c>
       <c r="L122" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M122" t="inlineStr"/>
       <c r="N122" t="n">
@@ -12979,7 +12979,7 @@
         <v>0</v>
       </c>
       <c r="L123" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M123" t="inlineStr"/>
       <c r="N123" t="n">
@@ -13083,7 +13083,7 @@
         <v>0</v>
       </c>
       <c r="L124" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M124" t="inlineStr"/>
       <c r="N124" t="n">
@@ -13187,7 +13187,7 @@
         <v>0</v>
       </c>
       <c r="L125" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M125" t="inlineStr"/>
       <c r="N125" t="n">
@@ -13291,7 +13291,7 @@
         <v>0</v>
       </c>
       <c r="L126" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M126" t="inlineStr"/>
       <c r="N126" t="n">
@@ -13395,7 +13395,7 @@
         <v>0</v>
       </c>
       <c r="L127" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M127" t="inlineStr"/>
       <c r="N127" t="n">
@@ -13499,7 +13499,7 @@
         <v>0</v>
       </c>
       <c r="L128" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M128" t="inlineStr"/>
       <c r="N128" t="n">
@@ -13603,7 +13603,7 @@
         <v>0</v>
       </c>
       <c r="L129" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M129" t="inlineStr"/>
       <c r="N129" t="n">
@@ -13707,7 +13707,7 @@
         <v>0</v>
       </c>
       <c r="L130" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M130" t="inlineStr"/>
       <c r="N130" t="n">
@@ -13811,7 +13811,7 @@
         <v>0</v>
       </c>
       <c r="L131" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M131" t="inlineStr"/>
       <c r="N131" t="n">
@@ -13915,7 +13915,7 @@
         <v>0</v>
       </c>
       <c r="L132" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M132" t="inlineStr"/>
       <c r="N132" t="n">
@@ -14019,7 +14019,7 @@
         <v>0</v>
       </c>
       <c r="L133" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M133" t="inlineStr"/>
       <c r="N133" t="n">
@@ -14123,7 +14123,7 @@
         <v>0</v>
       </c>
       <c r="L134" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M134" t="inlineStr"/>
       <c r="N134" t="n">
@@ -14227,7 +14227,7 @@
         <v>0</v>
       </c>
       <c r="L135" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M135" t="inlineStr"/>
       <c r="N135" t="n">
@@ -14331,7 +14331,7 @@
         <v>0</v>
       </c>
       <c r="L136" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M136" t="inlineStr"/>
       <c r="N136" t="n">
@@ -14435,7 +14435,7 @@
         <v>0</v>
       </c>
       <c r="L137" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M137" t="inlineStr"/>
       <c r="N137" t="n">
@@ -14539,7 +14539,7 @@
         <v>0</v>
       </c>
       <c r="L138" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M138" t="inlineStr"/>
       <c r="N138" t="n">
@@ -14643,7 +14643,7 @@
         <v>0</v>
       </c>
       <c r="L139" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M139" t="inlineStr"/>
       <c r="N139" t="n">
@@ -14747,7 +14747,7 @@
         <v>0</v>
       </c>
       <c r="L140" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M140" t="inlineStr"/>
       <c r="N140" t="n">
@@ -14851,7 +14851,7 @@
         <v>0</v>
       </c>
       <c r="L141" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M141" t="inlineStr"/>
       <c r="N141" t="n">
@@ -14955,7 +14955,7 @@
         <v>0</v>
       </c>
       <c r="L142" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M142" t="inlineStr"/>
       <c r="N142" t="n">
@@ -15059,7 +15059,7 @@
         <v>0</v>
       </c>
       <c r="L143" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M143" t="inlineStr"/>
       <c r="N143" t="n">
@@ -15163,7 +15163,7 @@
         <v>0</v>
       </c>
       <c r="L144" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="M144" t="inlineStr"/>
       <c r="N144" t="n">

</xml_diff>